<commit_message>
added endpoint ref status hidup
</commit_message>
<xml_diff>
--- a/ref/progress.xlsx
+++ b/ref/progress.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dinaskominfo/kiken/Project/next/e-office2026/ref/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6A804E67-B8A7-4144-B01F-0613D9F26E9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60AF45AF-6178-A948-A75F-99955B96C515}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="1000" windowWidth="27640" windowHeight="15300" xr2:uid="{B48B6E4E-04F9-0B46-B445-3CEA96597E01}"/>
+    <workbookView xWindow="6160" yWindow="1000" windowWidth="27640" windowHeight="15300" xr2:uid="{B48B6E4E-04F9-0B46-B445-3CEA96597E01}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -971,7 +971,7 @@
       </c>
     </row>
     <row r="18" spans="1:1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A18" s="1" t="s">
+      <c r="A18" s="6" t="s">
         <v>17</v>
       </c>
     </row>
@@ -986,7 +986,7 @@
       </c>
     </row>
     <row r="21" spans="1:1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A21" s="1" t="s">
+      <c r="A21" s="6" t="s">
         <v>20</v>
       </c>
     </row>
@@ -1221,22 +1221,22 @@
       </c>
     </row>
     <row r="68" spans="1:1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A68" s="1" t="s">
+      <c r="A68" s="6" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="69" spans="1:1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A69" s="1" t="s">
+      <c r="A69" s="6" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="70" spans="1:1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A70" s="1" t="s">
+      <c r="A70" s="6" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="71" spans="1:1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A71" s="1" t="s">
+      <c r="A71" s="6" t="s">
         <v>68</v>
       </c>
     </row>
@@ -1306,12 +1306,12 @@
       </c>
     </row>
     <row r="85" spans="1:1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A85" s="1" t="s">
+      <c r="A85" s="6" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="86" spans="1:1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A86" s="1" t="s">
+      <c r="A86" s="6" t="s">
         <v>83</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added crud ref jns lokasi
</commit_message>
<xml_diff>
--- a/ref/progress.xlsx
+++ b/ref/progress.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dinaskominfo/kiken/Project/next/e-office2026/ref/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60AF45AF-6178-A948-A75F-99955B96C515}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79F6F5AF-5B7C-A641-B7B0-A022D4ABDA03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6160" yWindow="1000" windowWidth="27640" windowHeight="15300" xr2:uid="{B48B6E4E-04F9-0B46-B445-3CEA96597E01}"/>
   </bookViews>
@@ -1031,22 +1031,22 @@
       </c>
     </row>
     <row r="30" spans="1:1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A30" s="1" t="s">
+      <c r="A30" s="5" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="31" spans="1:1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A31" s="1" t="s">
+      <c r="A31" s="5" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="32" spans="1:1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A32" s="1" t="s">
+      <c r="A32" s="5" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="33" spans="1:1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A33" s="1" t="s">
+      <c r="A33" s="5" t="s">
         <v>32</v>
       </c>
     </row>
@@ -1196,17 +1196,17 @@
       </c>
     </row>
     <row r="63" spans="1:1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A63" s="1" t="s">
+      <c r="A63" s="5" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="64" spans="1:1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A64" s="1" t="s">
+      <c r="A64" s="5" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="65" spans="1:1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A65" s="1" t="s">
+      <c r="A65" s="2" t="s">
         <v>62</v>
       </c>
     </row>
@@ -1316,7 +1316,7 @@
       </c>
     </row>
     <row r="87" spans="1:1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A87" s="1" t="s">
+      <c r="A87" s="6" t="s">
         <v>84</v>
       </c>
     </row>
@@ -1466,7 +1466,7 @@
       </c>
     </row>
     <row r="117" spans="1:1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A117" s="1" t="s">
+      <c r="A117" s="2" t="s">
         <v>114</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added comment ref KPPN
</commit_message>
<xml_diff>
--- a/ref/progress.xlsx
+++ b/ref/progress.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dinaskominfo/kiken/Project/next/e-office2026/ref/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79F6F5AF-5B7C-A641-B7B0-A022D4ABDA03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{054CD756-FA39-9F47-B581-D468B9EC2E61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6160" yWindow="1000" windowWidth="27640" windowHeight="15300" xr2:uid="{B48B6E4E-04F9-0B46-B445-3CEA96597E01}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15800" xr2:uid="{B48B6E4E-04F9-0B46-B445-3CEA96597E01}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -921,12 +921,12 @@
       </c>
     </row>
     <row r="8" spans="1:1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
     </row>
@@ -1086,22 +1086,22 @@
       </c>
     </row>
     <row r="41" spans="1:1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A41" s="1" t="s">
+      <c r="A41" s="5" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="42" spans="1:1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A42" s="1" t="s">
+      <c r="A42" s="5" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="43" spans="1:1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A43" s="1" t="s">
+      <c r="A43" s="5" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="44" spans="1:1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A44" s="1" t="s">
+      <c r="A44" s="5" t="s">
         <v>43</v>
       </c>
     </row>
@@ -1211,12 +1211,12 @@
       </c>
     </row>
     <row r="66" spans="1:1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A66" s="1" t="s">
+      <c r="A66" s="5" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="67" spans="1:1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A67" s="1" t="s">
+      <c r="A67" s="5" t="s">
         <v>64</v>
       </c>
     </row>

</xml_diff>